<commit_message>
First pass at public reflex site
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@149 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC ERD.xlsx
+++ b/Documentation/LRC ERD.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pype\cola\lrc-site\Documentation\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11805" windowHeight="5145"/>
   </bookViews>
@@ -4300,7 +4295,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4308,11 +4303,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="70" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Etymas – loaded HTML instead of just text to capture bolds Etyma Glosses loaded with HTML because some have bols Sub Fams loaded with HTML because some have bolds Changed language loaded to handle case where a lang doesn’t have a subfamily.  Create a subfamily called ‘’ – Changed lang page to match Added family override switch to language and changed reflex page to use it 		Created reflex entry table so that a reflex can be made up of more than one word.  Changed reflex and lang reflex to use this 		Changed lang reflex page to turn reflexes with () into to reflexes. 		Changed lang reflex page to combine 2 reflexes if they are the same and list their etyma together.  Even though their gloss and pos may be different 		Changed ReflexPOS to store their reflex and use POS table as a lookup 	Tested FacDB and Scholarships to make sure updates to Tomcat haven’t affected them
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@154 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC ERD.xlsx
+++ b/Documentation/LRC ERD.xlsx
@@ -1053,13 +1053,6 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1000" baseline="0"/>
-            <a:t>reflex</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0">
               <a:solidFill>
@@ -1475,7 +1468,7 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>498400</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>121834</xdr:rowOff>
+      <xdr:rowOff>13804</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
@@ -1490,8 +1483,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4142748" y="4953356"/>
-          <a:ext cx="1357000" cy="1300014"/>
+          <a:off x="4142748" y="4845326"/>
+          <a:ext cx="1357000" cy="1408044"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1566,6 +1559,13 @@
             <a:t>Sub Family ID</a:t>
           </a:r>
         </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" baseline="0"/>
+            <a:t>Override Family</a:t>
+          </a:r>
+        </a:p>
       </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
@@ -1575,7 +1575,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>487325</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>192059</xdr:rowOff>
+      <xdr:rowOff>138044</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
@@ -1593,8 +1593,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="3524282" y="5603363"/>
-          <a:ext cx="618466" cy="1069675"/>
+          <a:off x="3524282" y="5549348"/>
+          <a:ext cx="618466" cy="1123690"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3833,7 +3833,7 @@
           <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1000" baseline="0"/>
-            <a:t>Part of Speech ID</a:t>
+            <a:t>Text</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -4012,6 +4012,139 @@
         <a:xfrm flipH="1" flipV="1">
           <a:off x="1529554" y="5943746"/>
           <a:ext cx="323853" cy="729292"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>41413</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>151847</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>221280</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>91493</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="Rectangle 57"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1863587" y="8075543"/>
+          <a:ext cx="1394650" cy="905950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" b="1" u="sng"/>
+            <a:t>Lex </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" b="1" u="sng" baseline="0"/>
+            <a:t> Reflex_Entry</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1000" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" baseline="0"/>
+            <a:t>ID</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" baseline="0"/>
+            <a:t>Reflex ID</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" baseline="0"/>
+            <a:t>Entry</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>131347</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>259280</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>151847</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="63" name="Straight Arrow Connector 62"/>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="14" idx="2"/>
+          <a:endCxn id="58" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="2560912" y="7343913"/>
+          <a:ext cx="127933" cy="731630"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4295,7 +4428,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
Tweaked language page to handle two () in one entry using recursion.  Better load entries.  Make Lang-reflex page more efficeint by using sql instead of eloquent orm.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@155 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC ERD.xlsx
+++ b/Documentation/LRC ERD.xlsx
@@ -4040,15 +4040,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>41413</xdr:colOff>
+      <xdr:colOff>151848</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>151847</xdr:rowOff>
+      <xdr:rowOff>165652</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>221280</xdr:colOff>
+      <xdr:colOff>331715</xdr:colOff>
       <xdr:row>46</xdr:row>
-      <xdr:rowOff>91493</xdr:rowOff>
+      <xdr:rowOff>105298</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -4057,7 +4057,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1863587" y="8075543"/>
+          <a:off x="1974022" y="8089348"/>
           <a:ext cx="1394650" cy="905950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4123,7 +4123,7 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>131347</xdr:colOff>
+      <xdr:colOff>241782</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -4131,7 +4131,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>259280</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>151847</xdr:rowOff>
+      <xdr:rowOff>165652</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -4143,8 +4143,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="2560912" y="7343913"/>
-          <a:ext cx="127933" cy="731630"/>
+          <a:off x="2671347" y="7343913"/>
+          <a:ext cx="17498" cy="745435"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4428,7 +4428,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
fixed up the clickable glosses.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@162 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC ERD.xlsx
+++ b/Documentation/LRC ERD.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fmcgrath\workspace\lrc-site\Documentation\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
   </bookViews>
@@ -2508,10 +2503,10 @@
           <a:r>
             <a:rPr lang="en-US" sz="1000" baseline="0">
               <a:solidFill>
-                <a:srgbClr val="FF0000"/>
+                <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Etyma ID - add later</a:t>
+            <a:t>Etyma ID</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -4433,7 +4428,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
added author and admin comments to lesson.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@235 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC ERD.xlsx
+++ b/Documentation/LRC ERD.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fmcgrath\workspace\lrc-site\Documentation\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="152511" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4428,7 +4433,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>